<commit_message>
docs: 4th IAA100 found (with 200 kg DYMH-103); parts-to-buy without amplifier
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parts-to-buy.xlsx
+++ b/docs/parts-to-buy.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>USD 60-130 (AliExpress / eBay); no EUR shop price found</t>
+          <t>ONLY if the found 200 kg cell fails the calibration check. USD 60-130 (AliExpress / eBay)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -634,65 +634,28 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Load-cell amplifier</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Futek IAA100 (FSH03863)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>871</v>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Elkome (EU)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>https://shop.elkome.com/en/iaa100-fsh03863-load-cell-amplifier</t>
-        </is>
-      </c>
-      <c r="H8" s="4">
-        <f>C8*D8</f>
+    <row r="9">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="H9" s="8">
+        <f>SUM(H5:H7)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="H10" s="8">
-        <f>SUM(H5:H8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="G11" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Note: maxon prices are excl. VAT; check VAT basis of the others</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Before ordering the ESCON: finish its meter tests (docs/tests/broken-tower-diagnosis.md, 2b3-2b12); only buy it if a test fails. New IAA100: copy a working module's DIP settings, trim to 0-3.3 V = 0-200 N.</t>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Before ordering the ESCON: finish its meter tests (docs/tests/broken-tower-diagnosis.md, 2b3-2b12); only buy it if a test fails. IAA100 not needed: 4th amplifier found 2026-10-05 (paired with a 200 kg, 1.0 mV/V DYMH-103).</t>
         </is>
       </c>
     </row>
@@ -701,7 +664,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: ESCON replacement needed; German sources in parts-to-buy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parts-to-buy.xlsx
+++ b/docs/parts-to-buy.xlsx
@@ -481,6 +481,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -634,6 +635,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -652,10 +654,11 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Before ordering the ESCON: finish its meter tests (docs/tests/broken-tower-diagnosis.md, 2b3-2b12); only buy it if a test fails. IAA100 not needed: 4th amplifier found 2026-10-05 (paired with a 200 kg, 1.0 mV/V DYMH-103).</t>
+          <t>ESCON: needed. Front tower's ESCON has a faulty control side (USB + enable dead, power stage OK; docs/tests/broken-tower-diagnosis.md, 2026-10-07). Order from Germany: maxon shop (link) or Farnell DE 2452179 (de.farnell.com); maxon Germany: info.de@maxongroup.com, +49 89 420 493-0. IAA100 not needed: 4th amplifier found 2026-10-05 (paired with a 200 kg, 1.0 mV/V DYMH-103).</t>
         </is>
       </c>
     </row>

</xml_diff>